<commit_message>
languages: 全量重集成 9 语言修复后工作区 (fr/ru/de/es/pt/ko/ar/ya 对应各源仓 2026-09-15 修复提交)
</commit_message>
<xml_diff>
--- a/languages/es/output/import/西班牙语专八精通.xlsx
+++ b/languages/es/output/import/西班牙语专八精通.xlsx
@@ -21147,7 +21147,7 @@
       </c>
       <c r="B651" s="1" t="inlineStr">
         <is>
-          <t>[peˈlado] 去皮的&lt;名&gt;</t>
+          <t>[peˈlado] 秃头的&lt;名&gt;</t>
         </is>
       </c>
       <c r="C651" s="1" t="inlineStr">
@@ -21157,7 +21157,7 @@
       </c>
       <c r="D651" s="1" t="inlineStr">
         <is>
-          <t>去皮的</t>
+          <t>秃头的</t>
         </is>
       </c>
       <c r="E651" s="1" t="inlineStr">

</xml_diff>